<commit_message>
Added admin role access and database edits
</commit_message>
<xml_diff>
--- a/data/LoginInfo.xlsx
+++ b/data/LoginInfo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,11 @@
           <t>Password</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +454,45 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>$2b$10$4GpJI2wgDVqztM/YLBui2uVC323Fkjr.QOMbwRUJWvlkHuWKd1c0m</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>jerry</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$2b$10$JwCmsCvLBlF8eZpjUGyNFeqmf2BBkxQO3Fh0Q4dwzkuptmqOQZiVG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>newUser</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$2b$10$Yhzc.k.LBQT688zfbhKrOeVoQwVJoRTjs/Z0lMaXtDXG5Ria0QFGC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>user</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added security and fixed login issues
</commit_message>
<xml_diff>
--- a/data/LoginInfo.xlsx
+++ b/data/LoginInfo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,6 +491,40 @@
         </is>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Alexa</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$2b$10$vlu7ki3H9eCJUmddKzeIrOcE6aCK8G/LGXA7vZfsmps9KjScMW7W6</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$2b$10$IuCX9gWF1utcypewFjKwJOhwzt5zzChNCpy4jnFNG6lspF0eFRNQS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>user</t>
         </is>

</xml_diff>